<commit_message>
updated for consistency with delivery block in standard init file
</commit_message>
<xml_diff>
--- a/config/CalSim3GroundWaterDataExtractionInitFile_v1.xlsx
+++ b/config/CalSim3GroundWaterDataExtractionInitFile_v1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96085474-AFFF-4CE1-96C6-9795E96A376A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A635DADB-D218-4437-A709-D2731022414E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -225,9 +225,6 @@
     <t>SV Dss path names</t>
   </si>
   <si>
-    <t>O475</t>
-  </si>
-  <si>
     <t>E266</t>
   </si>
   <si>
@@ -250,6 +247,9 @@
   </si>
   <si>
     <t>J26</t>
+  </si>
+  <si>
+    <t>O472</t>
   </si>
 </sst>
 </file>
@@ -643,7 +643,7 @@
         <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E5" s="2"/>
     </row>
@@ -658,7 +658,7 @@
         <v>34</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E6" s="2"/>
     </row>
@@ -673,7 +673,7 @@
         <v>19</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E7" s="2"/>
     </row>
@@ -688,7 +688,7 @@
         <v>20</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E8" s="2"/>
     </row>
@@ -703,7 +703,7 @@
         <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E9" s="2"/>
     </row>
@@ -718,7 +718,7 @@
         <v>22</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E10" s="2"/>
     </row>
@@ -733,7 +733,7 @@
         <v>35</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E11" s="2"/>
     </row>
@@ -772,7 +772,7 @@
         <v>25</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -834,7 +834,7 @@
         <v>43</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>